<commit_message>
fix market context data fetch
</commit_message>
<xml_diff>
--- a/A股每日选股报告页面设计/public/reports/20260625/stock_pick_20260625.xlsx
+++ b/A股每日选股报告页面设计/public/reports/20260625/stock_pick_20260625.xlsx
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>107.01</v>
+        <v>107.81</v>
       </c>
       <c r="C5" s="5" t="inlineStr"/>
       <c r="D5" s="2" t="n"/>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>91.2705</v>
+        <v>91.0305</v>
       </c>
       <c r="C6" s="5" t="inlineStr"/>
       <c r="D6" s="2" t="n"/>
@@ -1101,10 +1101,10 @@
     <col width="8" customWidth="1" min="17" max="17"/>
     <col width="8" customWidth="1" min="18" max="18"/>
     <col width="8" customWidth="1" min="19" max="19"/>
-    <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
     <col width="9" customWidth="1" min="22" max="22"/>
-    <col width="23" customWidth="1" min="23" max="23"/>
+    <col width="28" customWidth="1" min="23" max="23"/>
     <col width="8" customWidth="1" min="24" max="24"/>
     <col width="8" customWidth="1" min="25" max="25"/>
     <col width="8" customWidth="1" min="26" max="26"/>
@@ -1390,7 +1390,7 @@
         <v>10.08</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>107.01</v>
+        <v>107.81</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>14.16</v>
@@ -1426,16 +1426,16 @@
         <v>9.75</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="T2" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>公告偏风险(2个负面关键词, 0个异动/风险词)</t>
         </is>
       </c>
       <c r="U2" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额上升2.9%</t>
         </is>
       </c>
       <c r="V2" s="4" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="W2" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>公告偏风险(2个负面关键词, 0个异动/风险词)；融资余额上升2.9%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X2" s="4" t="n">
@@ -1553,7 +1553,7 @@
         <v>6.6</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>101.06</v>
+        <v>99.26000000000001</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>15</v>
@@ -1589,16 +1589,16 @@
         <v>7.75</v>
       </c>
       <c r="S3" s="4" t="n">
-        <v>0</v>
+        <v>-1.8</v>
       </c>
       <c r="T3" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>近期公告中性</t>
         </is>
       </c>
       <c r="U3" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额下降-3.3%</t>
         </is>
       </c>
       <c r="V3" s="4" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="W3" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>近期公告中性；融资余额下降-3.3%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X3" s="4" t="n">
@@ -1716,7 +1716,7 @@
         <v>6.67</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>98.97</v>
+        <v>99.17</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>15</v>
@@ -1752,16 +1752,16 @@
         <v>7.88</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="T4" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>近期公告中性</t>
         </is>
       </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额上升3.0%</t>
         </is>
       </c>
       <c r="V4" s="4" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="W4" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>近期公告中性；融资余额上升3.0%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X4" s="4" t="n">
@@ -1919,22 +1919,22 @@
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="V5" s="4" t="inlineStr">
         <is>
-          <t>近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="W5" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="X5" s="4" t="n">
@@ -2042,7 +2042,7 @@
         <v>10</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>94.04000000000001</v>
+        <v>94.23999999999999</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>12.8</v>
@@ -2078,16 +2078,16 @@
         <v>9.31</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="T6" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>公告偏正面(4个积极关键词)</t>
         </is>
       </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额下降-12.6%</t>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="W6" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>公告偏正面(4个积极关键词)；融资余额下降-12.6%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X6" s="4" t="n">
@@ -2189,41 +2189,41 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>600058</t>
+          <t>601678</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>五矿发展</t>
+          <t>滨化股份</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="4" t="n">
-        <v>11.77</v>
+        <v>6.51</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>10</v>
+        <v>6.03</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>92.06999999999999</v>
+        <v>93.88</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>8.390000000000001</v>
+        <v>12.47</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>-0.2231</v>
+        <v>1.6623</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>1.144329</v>
+        <v>1.126395</v>
       </c>
       <c r="L7" s="4" t="n">
-        <v>5.31</v>
+        <v>4.82</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>14.93</v>
+        <v>11.79</v>
       </c>
       <c r="N7" s="4" t="n">
         <v>8</v>
@@ -2232,25 +2232,25 @@
         <v>10</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>16.32</v>
+        <v>19.62</v>
       </c>
       <c r="Q7" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="R7" s="4" t="n">
-        <v>9.119999999999999</v>
+        <v>7.38</v>
       </c>
       <c r="S7" s="4" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="T7" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>近期公告中性</t>
         </is>
       </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额上升7.0%</t>
         </is>
       </c>
       <c r="V7" s="4" t="inlineStr">
@@ -2260,29 +2260,29 @@
       </c>
       <c r="W7" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>近期公告中性；融资余额上升7.0%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X7" s="4" t="n">
-        <v>44.9</v>
+        <v>38.6</v>
       </c>
       <c r="Y7" s="4" t="n">
-        <v>37.03</v>
+        <v>35.25</v>
       </c>
       <c r="Z7" s="4" t="n">
-        <v>10.39</v>
+        <v>11.74</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>1.33</v>
+        <v>1.21</v>
       </c>
       <c r="AB7" s="4" t="n">
-        <v>0.115259</v>
+        <v>0.145687</v>
       </c>
       <c r="AC7" s="4" t="n">
-        <v>0.08749999999999999</v>
+        <v>0.2625</v>
       </c>
       <c r="AD7" s="4" t="n">
-        <v>0.08749999999999999</v>
+        <v>0.2625</v>
       </c>
       <c r="AE7" s="4" t="inlineStr">
         <is>
@@ -2293,56 +2293,56 @@
         <v>3</v>
       </c>
       <c r="AG7" s="4" t="n">
-        <v>10.95</v>
+        <v>6.05</v>
       </c>
       <c r="AH7" s="4" t="n">
-        <v>13.09</v>
+        <v>7.24</v>
       </c>
       <c r="AI7" s="4" t="n">
-        <v>13.95</v>
+        <v>7.69</v>
       </c>
       <c r="AJ7" s="4" t="n">
-        <v>10.95</v>
+        <v>6.08</v>
       </c>
       <c r="AK7" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL7" s="4" t="inlineStr">
         <is>
-          <t>3日短线计划；T+1看12.51/止损11.36；T+2看12.76/止损10.95；T+3看13.09/止损10.95</t>
+          <t>3日短线计划；T+1看6.92/止损6.28；T+2看7.06/止损6.11；T+3看7.24/止损6.08</t>
         </is>
       </c>
       <c r="AM7" s="4" t="n">
-        <v>11.36</v>
+        <v>6.28</v>
       </c>
       <c r="AN7" s="4" t="n">
-        <v>12.51</v>
+        <v>6.92</v>
       </c>
       <c r="AO7" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到12.51先减仓，跌破11.36止损；若高开低走不恋战</t>
+          <t>T+1：冲到6.92先减仓，跌破6.28止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP7" s="4" t="n">
-        <v>10.95</v>
+        <v>6.11</v>
       </c>
       <c r="AQ7" s="4" t="n">
-        <v>12.76</v>
+        <v>7.06</v>
       </c>
       <c r="AR7" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破12.76且量能转弱则减仓，跌破10.95退出</t>
+          <t>T+2：未突破7.06且量能转弱则减仓，跌破6.11退出</t>
         </is>
       </c>
       <c r="AS7" s="4" t="n">
-        <v>10.95</v>
+        <v>6.08</v>
       </c>
       <c r="AT7" s="4" t="n">
-        <v>13.09</v>
+        <v>7.24</v>
       </c>
       <c r="AU7" s="4" t="inlineStr">
         <is>
-          <t>T+3：到13.09分批止盈，跌破10.95或MA5失守退出</t>
+          <t>T+3：到7.24分批止盈，跌破6.08或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2352,41 +2352,41 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>601678</t>
+          <t>600058</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>滨化股份</t>
+          <t>五矿发展</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="4" t="n">
-        <v>6.51</v>
+        <v>11.77</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>6.03</v>
+        <v>10</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>91.08</v>
+        <v>90.27</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>12.47</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>1.6623</v>
+        <v>-0.2231</v>
       </c>
       <c r="K8" s="4" t="n">
-        <v>1.126395</v>
+        <v>1.144329</v>
       </c>
       <c r="L8" s="4" t="n">
-        <v>4.82</v>
+        <v>5.31</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>11.79</v>
+        <v>14.93</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>8</v>
@@ -2395,25 +2395,25 @@
         <v>10</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>19.62</v>
+        <v>16.32</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R8" s="4" t="n">
-        <v>7.38</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="S8" s="4" t="n">
-        <v>0</v>
+        <v>-1.8</v>
       </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>近期公告中性</t>
         </is>
       </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额下降-1.9%</t>
         </is>
       </c>
       <c r="V8" s="4" t="inlineStr">
@@ -2423,29 +2423,29 @@
       </c>
       <c r="W8" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>近期公告中性；融资余额下降-1.9%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X8" s="4" t="n">
-        <v>38.6</v>
+        <v>44.9</v>
       </c>
       <c r="Y8" s="4" t="n">
-        <v>35.25</v>
+        <v>37.03</v>
       </c>
       <c r="Z8" s="4" t="n">
-        <v>11.74</v>
+        <v>10.39</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>1.21</v>
+        <v>1.33</v>
       </c>
       <c r="AB8" s="4" t="n">
-        <v>0.145687</v>
+        <v>0.115259</v>
       </c>
       <c r="AC8" s="4" t="n">
-        <v>0.2625</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="AD8" s="4" t="n">
-        <v>0.2625</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="AE8" s="4" t="inlineStr">
         <is>
@@ -2456,56 +2456,56 @@
         <v>3</v>
       </c>
       <c r="AG8" s="4" t="n">
-        <v>6.05</v>
+        <v>10.95</v>
       </c>
       <c r="AH8" s="4" t="n">
-        <v>7.24</v>
+        <v>13.09</v>
       </c>
       <c r="AI8" s="4" t="n">
-        <v>7.69</v>
+        <v>13.95</v>
       </c>
       <c r="AJ8" s="4" t="n">
-        <v>6.08</v>
+        <v>10.95</v>
       </c>
       <c r="AK8" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL8" s="4" t="inlineStr">
         <is>
-          <t>3日短线计划；T+1看6.92/止损6.28；T+2看7.06/止损6.11；T+3看7.24/止损6.08</t>
+          <t>3日短线计划；T+1看12.51/止损11.36；T+2看12.76/止损10.95；T+3看13.09/止损10.95</t>
         </is>
       </c>
       <c r="AM8" s="4" t="n">
-        <v>6.28</v>
+        <v>11.36</v>
       </c>
       <c r="AN8" s="4" t="n">
-        <v>6.92</v>
+        <v>12.51</v>
       </c>
       <c r="AO8" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到6.92先减仓，跌破6.28止损；若高开低走不恋战</t>
+          <t>T+1：冲到12.51先减仓，跌破11.36止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP8" s="4" t="n">
-        <v>6.11</v>
+        <v>10.95</v>
       </c>
       <c r="AQ8" s="4" t="n">
-        <v>7.06</v>
+        <v>12.76</v>
       </c>
       <c r="AR8" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破7.06且量能转弱则减仓，跌破6.11退出</t>
+          <t>T+2：未突破12.76且量能转弱则减仓，跌破10.95退出</t>
         </is>
       </c>
       <c r="AS8" s="4" t="n">
-        <v>6.08</v>
+        <v>10.95</v>
       </c>
       <c r="AT8" s="4" t="n">
-        <v>7.24</v>
+        <v>13.09</v>
       </c>
       <c r="AU8" s="4" t="inlineStr">
         <is>
-          <t>T+3：到7.24分批止盈，跌破6.08或MA5失守退出</t>
+          <t>T+3：到13.09分批止盈，跌破10.95或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
         <v>4.27</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>90.8</v>
+        <v>90</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>14.97</v>
@@ -2567,16 +2567,16 @@
         <v>6</v>
       </c>
       <c r="S9" s="4" t="n">
-        <v>0</v>
+        <v>-0.8</v>
       </c>
       <c r="T9" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>近期公告中性</t>
         </is>
       </c>
       <c r="U9" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额下降-0.8%</t>
         </is>
       </c>
       <c r="V9" s="4" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="W9" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>近期公告中性；融资余额下降-0.8%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X9" s="4" t="n">
@@ -2734,22 +2734,22 @@
       </c>
       <c r="T10" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="V10" s="4" t="inlineStr">
         <is>
-          <t>近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="W10" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="X10" s="4" t="n">
@@ -2841,100 +2841,100 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>000100</t>
+          <t>000766</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>TCL科技</t>
+          <t>通化金马</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="4" t="n">
-        <v>5.34</v>
+        <v>26.61</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>89.7</v>
+        <v>89.66</v>
       </c>
       <c r="H11" s="4" t="n">
         <v>15</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>5.2684</v>
+        <v>3.4775</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>1.125277</v>
+        <v>1.085259</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>5.84</v>
+        <v>10</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>9.449999999999999</v>
+        <v>7.43</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="O11" s="4" t="n">
-        <v>10</v>
+        <v>5.25</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>4.53</v>
+        <v>14.67</v>
       </c>
       <c r="Q11" s="4" t="n">
         <v>20</v>
       </c>
       <c r="R11" s="4" t="n">
-        <v>9.880000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="S11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T11" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="U11" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="V11" s="4" t="inlineStr">
         <is>
-          <t>近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="W11" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="X11" s="4" t="n">
-        <v>33.9</v>
+        <v>29.9</v>
       </c>
       <c r="Y11" s="4" t="n">
-        <v>38.9</v>
+        <v>32.92</v>
       </c>
       <c r="Z11" s="4" t="n">
-        <v>13.38</v>
+        <v>11.1</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>1.46</v>
+        <v>3.78</v>
       </c>
       <c r="AB11" s="4" t="n">
-        <v>0.00655</v>
+        <v>0.100062</v>
       </c>
       <c r="AC11" s="4" t="n">
-        <v>0.0125</v>
+        <v>0.0688</v>
       </c>
       <c r="AD11" s="4" t="n">
-        <v>0.0125</v>
+        <v>0.0688</v>
       </c>
       <c r="AE11" s="4" t="inlineStr">
         <is>
@@ -2945,56 +2945,56 @@
         <v>2</v>
       </c>
       <c r="AG11" s="4" t="n">
-        <v>4.97</v>
+        <v>24.95</v>
       </c>
       <c r="AH11" s="4" t="n">
-        <v>5.94</v>
+        <v>29.26</v>
       </c>
       <c r="AI11" s="4" t="n">
-        <v>6.31</v>
+        <v>30.92</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>5.01</v>
+        <v>25.5</v>
       </c>
       <c r="AK11" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL11" s="4" t="inlineStr">
         <is>
-          <t>2日短线计划；T+1看5.68/止损5.15；T+2看5.79/止损4.98；T+3看5.94/止损5.01</t>
+          <t>2日短线计划；T+1看28.10/止损25.69；T+2看28.60/止损25.41；T+3看29.26/止损25.50</t>
         </is>
       </c>
       <c r="AM11" s="4" t="n">
-        <v>5.15</v>
+        <v>25.69</v>
       </c>
       <c r="AN11" s="4" t="n">
-        <v>5.68</v>
+        <v>28.1</v>
       </c>
       <c r="AO11" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到5.68先减仓，跌破5.15止损；若高开低走不恋战</t>
+          <t>T+1：冲到28.10先减仓，跌破25.69止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP11" s="4" t="n">
-        <v>4.98</v>
+        <v>25.41</v>
       </c>
       <c r="AQ11" s="4" t="n">
-        <v>5.79</v>
+        <v>28.6</v>
       </c>
       <c r="AR11" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破5.79且量能转弱则减仓，跌破4.98退出</t>
+          <t>T+2：未突破28.60且量能转弱则减仓，跌破25.41退出</t>
         </is>
       </c>
       <c r="AS11" s="4" t="n">
-        <v>5.01</v>
+        <v>25.5</v>
       </c>
       <c r="AT11" s="4" t="n">
-        <v>5.94</v>
+        <v>29.26</v>
       </c>
       <c r="AU11" s="4" t="inlineStr">
         <is>
-          <t>T+3：到5.94分批止盈，跌破5.01或MA5失守退出</t>
+          <t>T+3：到29.26分批止盈，跌破25.50或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3004,160 +3004,160 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>000766</t>
+          <t>000783</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>通化金马</t>
+          <t>长江证券</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="4" t="n">
-        <v>26.61</v>
+        <v>10.15</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>10</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>89.66</v>
+        <v>89.59</v>
       </c>
       <c r="H12" s="4" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0.2668</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>1.256344</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>8.48</v>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>15</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>3.4775</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>1.085259</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>7.43</v>
       </c>
       <c r="N12" s="4" t="n">
         <v>8</v>
       </c>
       <c r="O12" s="4" t="n">
-        <v>5.25</v>
+        <v>10</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>14.67</v>
+        <v>18.1</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>20</v>
       </c>
       <c r="R12" s="4" t="n">
-        <v>9.31</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="S12" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T12" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="V12" s="4" t="inlineStr">
         <is>
-          <t>近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="W12" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="X12" s="4" t="n">
-        <v>29.9</v>
+        <v>53.6</v>
       </c>
       <c r="Y12" s="4" t="n">
-        <v>32.92</v>
+        <v>48.53</v>
       </c>
       <c r="Z12" s="4" t="n">
-        <v>11.1</v>
+        <v>4.93</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>3.78</v>
+        <v>2.12</v>
       </c>
       <c r="AB12" s="4" t="n">
-        <v>0.100062</v>
+        <v>0.131632</v>
       </c>
       <c r="AC12" s="4" t="n">
-        <v>0.0688</v>
+        <v>0.1125</v>
       </c>
       <c r="AD12" s="4" t="n">
-        <v>0.0688</v>
+        <v>0.1125</v>
       </c>
       <c r="AE12" s="4" t="inlineStr">
         <is>
-          <t>🟡 首日上涨，可关注</t>
+          <t>🟠 远离均线，不宜追高</t>
         </is>
       </c>
       <c r="AF12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG12" s="4" t="n">
-        <v>24.95</v>
+        <v>9.44</v>
       </c>
       <c r="AH12" s="4" t="n">
-        <v>29.26</v>
+        <v>11.29</v>
       </c>
       <c r="AI12" s="4" t="n">
-        <v>30.92</v>
+        <v>12</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>25.5</v>
+        <v>9.59</v>
       </c>
       <c r="AK12" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL12" s="4" t="inlineStr">
         <is>
-          <t>2日短线计划；T+1看28.10/止损25.69；T+2看28.60/止损25.41；T+3看29.26/止损25.50</t>
+          <t>1日短线计划；T+1看10.79/止损9.79；T+2看11.00/止损9.54；T+3看11.29/止损9.59</t>
         </is>
       </c>
       <c r="AM12" s="4" t="n">
-        <v>25.69</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="AN12" s="4" t="n">
-        <v>28.1</v>
+        <v>10.79</v>
       </c>
       <c r="AO12" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到28.10先减仓，跌破25.69止损；若高开低走不恋战</t>
+          <t>T+1：冲到10.79先减仓，跌破9.79止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP12" s="4" t="n">
-        <v>25.41</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="AQ12" s="4" t="n">
-        <v>28.6</v>
+        <v>11</v>
       </c>
       <c r="AR12" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破28.60且量能转弱则减仓，跌破25.41退出</t>
+          <t>T+2：未突破11.00且量能转弱则减仓，跌破9.54退出</t>
         </is>
       </c>
       <c r="AS12" s="4" t="n">
-        <v>25.5</v>
+        <v>9.59</v>
       </c>
       <c r="AT12" s="4" t="n">
-        <v>29.26</v>
+        <v>11.29</v>
       </c>
       <c r="AU12" s="4" t="inlineStr">
         <is>
-          <t>T+3：到29.26分批止盈，跌破25.50或MA5失守退出</t>
+          <t>T+3：到11.29分批止盈，跌破9.59或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3167,38 +3167,38 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>000783</t>
+          <t>000021</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>长江证券</t>
+          <t>深科技</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="4" t="n">
-        <v>10.15</v>
+        <v>53.2</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>9.970000000000001</v>
+        <v>5.83</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>89.59</v>
+        <v>89.33</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>5.13</v>
+        <v>13.1</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.2668</v>
+        <v>7.3979</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>1.256344</v>
+        <v>1.293082</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>8.48</v>
+        <v>4.91</v>
       </c>
       <c r="M13" s="4" t="n">
         <v>15</v>
@@ -3210,57 +3210,57 @@
         <v>10</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>18.1</v>
+        <v>20.2</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="R13" s="4" t="n">
-        <v>8.880000000000001</v>
+        <v>7.12</v>
       </c>
       <c r="S13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T13" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="U13" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="V13" s="4" t="inlineStr">
         <is>
-          <t>近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="W13" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="X13" s="4" t="n">
-        <v>53.6</v>
+        <v>54.8</v>
       </c>
       <c r="Y13" s="4" t="n">
-        <v>48.53</v>
+        <v>46.5</v>
       </c>
       <c r="Z13" s="4" t="n">
-        <v>4.93</v>
+        <v>4.28</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>2.12</v>
+        <v>1.23</v>
       </c>
       <c r="AB13" s="4" t="n">
-        <v>0.131632</v>
+        <v>0.151</v>
       </c>
       <c r="AC13" s="4" t="n">
-        <v>0.1125</v>
+        <v>0.2875</v>
       </c>
       <c r="AD13" s="4" t="n">
-        <v>0.1125</v>
+        <v>0.2875</v>
       </c>
       <c r="AE13" s="4" t="inlineStr">
         <is>
@@ -3271,56 +3271,56 @@
         <v>1</v>
       </c>
       <c r="AG13" s="4" t="n">
-        <v>9.44</v>
+        <v>49.48</v>
       </c>
       <c r="AH13" s="4" t="n">
-        <v>11.29</v>
+        <v>59.16</v>
       </c>
       <c r="AI13" s="4" t="n">
-        <v>12</v>
+        <v>62.99</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>9.59</v>
+        <v>49.48</v>
       </c>
       <c r="AK13" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL13" s="4" t="inlineStr">
         <is>
-          <t>1日短线计划；T+1看10.79/止损9.79；T+2看11.00/止损9.54；T+3看11.29/止损9.59</t>
+          <t>1日短线计划；T+1看56.55/止损51.34；T+2看57.67/止损49.48；T+3看59.16/止损49.48</t>
         </is>
       </c>
       <c r="AM13" s="4" t="n">
-        <v>9.789999999999999</v>
+        <v>51.34</v>
       </c>
       <c r="AN13" s="4" t="n">
-        <v>10.79</v>
+        <v>56.55</v>
       </c>
       <c r="AO13" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到10.79先减仓，跌破9.79止损；若高开低走不恋战</t>
+          <t>T+1：冲到56.55先减仓，跌破51.34止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP13" s="4" t="n">
-        <v>9.539999999999999</v>
+        <v>49.48</v>
       </c>
       <c r="AQ13" s="4" t="n">
-        <v>11</v>
+        <v>57.67</v>
       </c>
       <c r="AR13" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破11.00且量能转弱则减仓，跌破9.54退出</t>
+          <t>T+2：未突破57.67且量能转弱则减仓，跌破49.48退出</t>
         </is>
       </c>
       <c r="AS13" s="4" t="n">
-        <v>9.59</v>
+        <v>49.48</v>
       </c>
       <c r="AT13" s="4" t="n">
-        <v>11.29</v>
+        <v>59.16</v>
       </c>
       <c r="AU13" s="4" t="inlineStr">
         <is>
-          <t>T+3：到11.29分批止盈，跌破9.59或MA5失守退出</t>
+          <t>T+3：到59.16分批止盈，跌破49.48或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3330,38 +3330,38 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>600141</t>
+          <t>601162</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>兴发集团</t>
+          <t>天风证券</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="4" t="n">
-        <v>47.48</v>
+        <v>3.59</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>10.01</v>
+        <v>4.36</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>89.37</v>
+        <v>89.31999999999999</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>11</v>
+        <v>8.52</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>10.9779</v>
+        <v>-3.0071</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>1.367906</v>
+        <v>1.091185</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>6.33</v>
+        <v>5.52</v>
       </c>
       <c r="M14" s="4" t="n">
         <v>15</v>
@@ -3370,28 +3370,28 @@
         <v>8</v>
       </c>
       <c r="O14" s="4" t="n">
-        <v>10</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>13.54</v>
+        <v>20.09</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="R14" s="4" t="n">
-        <v>9.5</v>
+        <v>6.12</v>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="T14" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>近期公告中性</t>
         </is>
       </c>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额上升1.2%</t>
         </is>
       </c>
       <c r="V14" s="4" t="inlineStr">
@@ -3401,89 +3401,89 @@
       </c>
       <c r="W14" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>近期公告中性；融资余额上升1.2%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X14" s="4" t="n">
-        <v>64.3</v>
+        <v>46.9</v>
       </c>
       <c r="Y14" s="4" t="n">
-        <v>51.55</v>
+        <v>37.32</v>
       </c>
       <c r="Z14" s="4" t="n">
-        <v>4.6</v>
+        <v>9.65</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>1.58</v>
+        <v>1.38</v>
       </c>
       <c r="AB14" s="4" t="n">
-        <v>0.08958099999999999</v>
+        <v>0.150034</v>
       </c>
       <c r="AC14" s="4" t="n">
-        <v>0.05</v>
+        <v>0.3875</v>
       </c>
       <c r="AD14" s="4" t="n">
-        <v>0.05</v>
+        <v>0.3875</v>
       </c>
       <c r="AE14" s="4" t="inlineStr">
         <is>
-          <t>🟠 远离均线，不宜追高</t>
+          <t>🟡 首日上涨，可关注</t>
         </is>
       </c>
       <c r="AF14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AG14" s="4" t="n">
-        <v>44.16</v>
+        <v>3.34</v>
       </c>
       <c r="AH14" s="4" t="n">
-        <v>52.8</v>
+        <v>3.99</v>
       </c>
       <c r="AI14" s="4" t="n">
-        <v>56.87</v>
+        <v>4.24</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>44.16</v>
+        <v>3.4</v>
       </c>
       <c r="AK14" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL14" s="4" t="inlineStr">
         <is>
-          <t>1日短线计划；T+1看50.47/止损45.82；T+2看51.47/止损44.16；T+3看52.80/止损44.16</t>
+          <t>3日短线计划；T+1看3.82/止损3.46；T+2看3.89/止损3.39；T+3看3.99/止损3.40</t>
         </is>
       </c>
       <c r="AM14" s="4" t="n">
-        <v>45.82</v>
+        <v>3.46</v>
       </c>
       <c r="AN14" s="4" t="n">
-        <v>50.47</v>
+        <v>3.82</v>
       </c>
       <c r="AO14" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到50.47先减仓，跌破45.82止损；若高开低走不恋战</t>
+          <t>T+1：冲到3.82先减仓，跌破3.46止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP14" s="4" t="n">
-        <v>44.16</v>
+        <v>3.39</v>
       </c>
       <c r="AQ14" s="4" t="n">
-        <v>51.47</v>
+        <v>3.89</v>
       </c>
       <c r="AR14" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破51.47且量能转弱则减仓，跌破44.16退出</t>
+          <t>T+2：未突破3.89且量能转弱则减仓，跌破3.39退出</t>
         </is>
       </c>
       <c r="AS14" s="4" t="n">
-        <v>44.16</v>
+        <v>3.4</v>
       </c>
       <c r="AT14" s="4" t="n">
-        <v>52.8</v>
+        <v>3.99</v>
       </c>
       <c r="AU14" s="4" t="inlineStr">
         <is>
-          <t>T+3：到52.80分批止盈，跌破44.16或MA5失守退出</t>
+          <t>T+3：到3.99分批止盈，跌破3.40或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3493,38 +3493,38 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>000021</t>
+          <t>600141</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>深科技</t>
+          <t>兴发集团</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="4" t="n">
-        <v>53.2</v>
+        <v>47.48</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>5.83</v>
+        <v>10.01</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>89.33</v>
+        <v>88.77</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>13.1</v>
+        <v>11</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>7.3979</v>
+        <v>10.9779</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>1.293082</v>
+        <v>1.367906</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>4.91</v>
+        <v>6.33</v>
       </c>
       <c r="M15" s="4" t="n">
         <v>15</v>
@@ -3536,25 +3536,25 @@
         <v>10</v>
       </c>
       <c r="P15" s="4" t="n">
-        <v>20.2</v>
+        <v>13.54</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R15" s="4" t="n">
-        <v>7.12</v>
+        <v>9.5</v>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="T15" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>公告偏风险(0个负面关键词, 1个异动/风险词)</t>
         </is>
       </c>
       <c r="U15" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额上升3.7%</t>
         </is>
       </c>
       <c r="V15" s="4" t="inlineStr">
@@ -3564,29 +3564,29 @@
       </c>
       <c r="W15" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>公告偏风险(0个负面关键词, 1个异动/风险词)；融资余额上升3.7%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X15" s="4" t="n">
-        <v>54.8</v>
+        <v>64.3</v>
       </c>
       <c r="Y15" s="4" t="n">
-        <v>46.5</v>
+        <v>51.55</v>
       </c>
       <c r="Z15" s="4" t="n">
-        <v>4.28</v>
+        <v>4.6</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>1.23</v>
+        <v>1.58</v>
       </c>
       <c r="AB15" s="4" t="n">
-        <v>0.151</v>
+        <v>0.08958099999999999</v>
       </c>
       <c r="AC15" s="4" t="n">
-        <v>0.2875</v>
+        <v>0.05</v>
       </c>
       <c r="AD15" s="4" t="n">
-        <v>0.2875</v>
+        <v>0.05</v>
       </c>
       <c r="AE15" s="4" t="inlineStr">
         <is>
@@ -3597,56 +3597,56 @@
         <v>1</v>
       </c>
       <c r="AG15" s="4" t="n">
-        <v>49.48</v>
+        <v>44.16</v>
       </c>
       <c r="AH15" s="4" t="n">
-        <v>59.16</v>
+        <v>52.8</v>
       </c>
       <c r="AI15" s="4" t="n">
-        <v>62.99</v>
+        <v>56.87</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>49.48</v>
+        <v>44.16</v>
       </c>
       <c r="AK15" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL15" s="4" t="inlineStr">
         <is>
-          <t>1日短线计划；T+1看56.55/止损51.34；T+2看57.67/止损49.48；T+3看59.16/止损49.48</t>
+          <t>1日短线计划；T+1看50.47/止损45.82；T+2看51.47/止损44.16；T+3看52.80/止损44.16</t>
         </is>
       </c>
       <c r="AM15" s="4" t="n">
-        <v>51.34</v>
+        <v>45.82</v>
       </c>
       <c r="AN15" s="4" t="n">
-        <v>56.55</v>
+        <v>50.47</v>
       </c>
       <c r="AO15" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到56.55先减仓，跌破51.34止损；若高开低走不恋战</t>
+          <t>T+1：冲到50.47先减仓，跌破45.82止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP15" s="4" t="n">
-        <v>49.48</v>
+        <v>44.16</v>
       </c>
       <c r="AQ15" s="4" t="n">
-        <v>57.67</v>
+        <v>51.47</v>
       </c>
       <c r="AR15" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破57.67且量能转弱则减仓，跌破49.48退出</t>
+          <t>T+2：未突破51.47且量能转弱则减仓，跌破44.16退出</t>
         </is>
       </c>
       <c r="AS15" s="4" t="n">
-        <v>49.48</v>
+        <v>44.16</v>
       </c>
       <c r="AT15" s="4" t="n">
-        <v>59.16</v>
+        <v>52.8</v>
       </c>
       <c r="AU15" s="4" t="inlineStr">
         <is>
-          <t>T+3：到59.16分批止盈，跌破49.48或MA5失守退出</t>
+          <t>T+3：到52.80分批止盈，跌破44.16或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3656,68 +3656,68 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>601162</t>
+          <t>000100</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>天风证券</t>
+          <t>TCL科技</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="4" t="n">
-        <v>3.59</v>
+        <v>5.34</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>4.36</v>
+        <v>10.1</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>89.12</v>
+        <v>88.5</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>8.52</v>
+        <v>15</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>-3.0071</v>
+        <v>5.2684</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>1.091185</v>
+        <v>1.125277</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>5.52</v>
+        <v>5.84</v>
       </c>
       <c r="M16" s="4" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="N16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="N16" s="4" t="n">
-        <v>8</v>
-      </c>
       <c r="O16" s="4" t="n">
-        <v>8.869999999999999</v>
+        <v>10</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>20.09</v>
+        <v>4.53</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R16" s="4" t="n">
-        <v>6.12</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="S16" s="4" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>公告偏风险(5个负面关键词, 0个异动/风险词)</t>
         </is>
       </c>
       <c r="U16" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额上升2.5%</t>
         </is>
       </c>
       <c r="V16" s="4" t="inlineStr">
@@ -3727,29 +3727,29 @@
       </c>
       <c r="W16" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>公告偏风险(5个负面关键词, 0个异动/风险词)；融资余额上升2.5%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X16" s="4" t="n">
-        <v>46.9</v>
+        <v>33.9</v>
       </c>
       <c r="Y16" s="4" t="n">
-        <v>37.32</v>
+        <v>38.9</v>
       </c>
       <c r="Z16" s="4" t="n">
-        <v>9.65</v>
+        <v>13.38</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>1.38</v>
+        <v>1.46</v>
       </c>
       <c r="AB16" s="4" t="n">
-        <v>0.150034</v>
+        <v>0.00655</v>
       </c>
       <c r="AC16" s="4" t="n">
-        <v>0.3875</v>
+        <v>0.0125</v>
       </c>
       <c r="AD16" s="4" t="n">
-        <v>0.3875</v>
+        <v>0.0125</v>
       </c>
       <c r="AE16" s="4" t="inlineStr">
         <is>
@@ -3757,59 +3757,59 @@
         </is>
       </c>
       <c r="AF16" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AG16" s="4" t="n">
-        <v>3.34</v>
+        <v>4.97</v>
       </c>
       <c r="AH16" s="4" t="n">
-        <v>3.99</v>
+        <v>5.94</v>
       </c>
       <c r="AI16" s="4" t="n">
-        <v>4.24</v>
+        <v>6.31</v>
       </c>
       <c r="AJ16" s="4" t="n">
-        <v>3.4</v>
+        <v>5.01</v>
       </c>
       <c r="AK16" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL16" s="4" t="inlineStr">
         <is>
-          <t>3日短线计划；T+1看3.82/止损3.46；T+2看3.89/止损3.39；T+3看3.99/止损3.40</t>
+          <t>2日短线计划；T+1看5.68/止损5.15；T+2看5.79/止损4.98；T+3看5.94/止损5.01</t>
         </is>
       </c>
       <c r="AM16" s="4" t="n">
-        <v>3.46</v>
+        <v>5.15</v>
       </c>
       <c r="AN16" s="4" t="n">
-        <v>3.82</v>
+        <v>5.68</v>
       </c>
       <c r="AO16" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到3.82先减仓，跌破3.46止损；若高开低走不恋战</t>
+          <t>T+1：冲到5.68先减仓，跌破5.15止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP16" s="4" t="n">
-        <v>3.39</v>
+        <v>4.98</v>
       </c>
       <c r="AQ16" s="4" t="n">
-        <v>3.89</v>
+        <v>5.79</v>
       </c>
       <c r="AR16" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破3.89且量能转弱则减仓，跌破3.39退出</t>
+          <t>T+2：未突破5.79且量能转弱则减仓，跌破4.98退出</t>
         </is>
       </c>
       <c r="AS16" s="4" t="n">
-        <v>3.4</v>
+        <v>5.01</v>
       </c>
       <c r="AT16" s="4" t="n">
-        <v>3.99</v>
+        <v>5.94</v>
       </c>
       <c r="AU16" s="4" t="inlineStr">
         <is>
-          <t>T+3：到3.99分批止盈，跌破3.40或MA5失守退出</t>
+          <t>T+3：到5.94分批止盈，跌破5.01或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -3875,22 +3875,22 @@
       </c>
       <c r="T17" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="U17" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="V17" s="4" t="inlineStr">
         <is>
-          <t>近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="W17" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="X17" s="4" t="n">
@@ -3982,41 +3982,41 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>600400</t>
+          <t>000066</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>红豆股份</t>
+          <t>中国长城</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="4" t="n">
-        <v>3.35</v>
+        <v>20.47</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>6.69</v>
+        <v>7.74</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>86.45999999999999</v>
+        <v>85.76000000000001</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>4.5</v>
+        <v>6.53</v>
       </c>
       <c r="I18" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>-3.0267</v>
+        <v>-7.6535</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>1.181449</v>
+        <v>1.170818</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>5.75</v>
+        <v>6.12</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>14.37</v>
+        <v>13.61</v>
       </c>
       <c r="N18" s="4" t="n">
         <v>8</v>
@@ -4025,57 +4025,57 @@
         <v>10</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>24.83</v>
+        <v>22.13</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>15</v>
       </c>
       <c r="R18" s="4" t="n">
-        <v>8</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="S18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="T18" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="V18" s="4" t="inlineStr">
         <is>
-          <t>近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="W18" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>上下文数据超时</t>
         </is>
       </c>
       <c r="X18" s="4" t="n">
-        <v>43.7</v>
+        <v>42.2</v>
       </c>
       <c r="Y18" s="4" t="n">
-        <v>39.95</v>
+        <v>38.71</v>
       </c>
       <c r="Z18" s="4" t="n">
-        <v>7.91</v>
+        <v>8.49</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>1.44</v>
+        <v>1.53</v>
       </c>
       <c r="AB18" s="4" t="n">
-        <v>0.193786</v>
+        <v>0.168841</v>
       </c>
       <c r="AC18" s="4" t="n">
-        <v>0.2</v>
+        <v>0.1625</v>
       </c>
       <c r="AD18" s="4" t="n">
-        <v>0.2</v>
+        <v>0.1625</v>
       </c>
       <c r="AE18" s="4" t="inlineStr">
         <is>
@@ -4086,56 +4086,56 @@
         <v>1</v>
       </c>
       <c r="AG18" s="4" t="n">
-        <v>3.12</v>
+        <v>19.04</v>
       </c>
       <c r="AH18" s="4" t="n">
-        <v>3.73</v>
+        <v>22.76</v>
       </c>
       <c r="AI18" s="4" t="n">
-        <v>3.96</v>
+        <v>24.2</v>
       </c>
       <c r="AJ18" s="4" t="n">
-        <v>3.12</v>
+        <v>19.14</v>
       </c>
       <c r="AK18" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL18" s="4" t="inlineStr">
         <is>
-          <t>1日短线计划；T+1看3.56/止损3.23；T+2看3.63/止损3.12；T+3看3.73/止损3.12</t>
+          <t>1日短线计划；T+1看21.76/止损19.75；T+2看22.19/止损19.04；T+3看22.76/止损19.14</t>
         </is>
       </c>
       <c r="AM18" s="4" t="n">
-        <v>3.23</v>
+        <v>19.75</v>
       </c>
       <c r="AN18" s="4" t="n">
-        <v>3.56</v>
+        <v>21.76</v>
       </c>
       <c r="AO18" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到3.56先减仓，跌破3.23止损；若高开低走不恋战</t>
+          <t>T+1：冲到21.76先减仓，跌破19.75止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP18" s="4" t="n">
-        <v>3.12</v>
+        <v>19.04</v>
       </c>
       <c r="AQ18" s="4" t="n">
-        <v>3.63</v>
+        <v>22.19</v>
       </c>
       <c r="AR18" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破3.63且量能转弱则减仓，跌破3.12退出</t>
+          <t>T+2：未突破22.19且量能转弱则减仓，跌破19.04退出</t>
         </is>
       </c>
       <c r="AS18" s="4" t="n">
-        <v>3.12</v>
+        <v>19.14</v>
       </c>
       <c r="AT18" s="4" t="n">
-        <v>3.73</v>
+        <v>22.76</v>
       </c>
       <c r="AU18" s="4" t="inlineStr">
         <is>
-          <t>T+3：到3.73分批止盈，跌破3.12或MA5失守退出</t>
+          <t>T+3：到22.76分批止盈，跌破19.14或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -4145,41 +4145,41 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>000066</t>
+          <t>600400</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>中国长城</t>
+          <t>红豆股份</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="4" t="n">
-        <v>20.47</v>
+        <v>3.35</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>7.74</v>
+        <v>6.69</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>85.76000000000001</v>
+        <v>84.66</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>6.53</v>
+        <v>4.5</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>-7.6535</v>
+        <v>-3.0267</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>1.170818</v>
+        <v>1.181449</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>6.12</v>
+        <v>5.75</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>13.61</v>
+        <v>14.37</v>
       </c>
       <c r="N19" s="4" t="n">
         <v>8</v>
@@ -4188,25 +4188,25 @@
         <v>10</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>22.13</v>
+        <v>24.83</v>
       </c>
       <c r="Q19" s="4" t="n">
         <v>15</v>
       </c>
       <c r="R19" s="4" t="n">
-        <v>8.380000000000001</v>
+        <v>8</v>
       </c>
       <c r="S19" s="4" t="n">
-        <v>0</v>
+        <v>-1.8</v>
       </c>
       <c r="T19" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>公告偏风险(2个负面关键词, 1个异动/风险词)</t>
         </is>
       </c>
       <c r="U19" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额上升16.3%</t>
         </is>
       </c>
       <c r="V19" s="4" t="inlineStr">
@@ -4216,29 +4216,29 @@
       </c>
       <c r="W19" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>公告偏风险(2个负面关键词, 1个异动/风险词)；融资余额上升16.3%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X19" s="4" t="n">
-        <v>42.2</v>
+        <v>43.7</v>
       </c>
       <c r="Y19" s="4" t="n">
-        <v>38.71</v>
+        <v>39.95</v>
       </c>
       <c r="Z19" s="4" t="n">
-        <v>8.49</v>
+        <v>7.91</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>1.53</v>
+        <v>1.44</v>
       </c>
       <c r="AB19" s="4" t="n">
-        <v>0.168841</v>
+        <v>0.193786</v>
       </c>
       <c r="AC19" s="4" t="n">
-        <v>0.1625</v>
+        <v>0.2</v>
       </c>
       <c r="AD19" s="4" t="n">
-        <v>0.1625</v>
+        <v>0.2</v>
       </c>
       <c r="AE19" s="4" t="inlineStr">
         <is>
@@ -4249,56 +4249,56 @@
         <v>1</v>
       </c>
       <c r="AG19" s="4" t="n">
-        <v>19.04</v>
+        <v>3.12</v>
       </c>
       <c r="AH19" s="4" t="n">
-        <v>22.76</v>
+        <v>3.73</v>
       </c>
       <c r="AI19" s="4" t="n">
-        <v>24.2</v>
+        <v>3.96</v>
       </c>
       <c r="AJ19" s="4" t="n">
-        <v>19.14</v>
+        <v>3.12</v>
       </c>
       <c r="AK19" s="4" t="n">
         <v>1.6</v>
       </c>
       <c r="AL19" s="4" t="inlineStr">
         <is>
-          <t>1日短线计划；T+1看21.76/止损19.75；T+2看22.19/止损19.04；T+3看22.76/止损19.14</t>
+          <t>1日短线计划；T+1看3.56/止损3.23；T+2看3.63/止损3.12；T+3看3.73/止损3.12</t>
         </is>
       </c>
       <c r="AM19" s="4" t="n">
-        <v>19.75</v>
+        <v>3.23</v>
       </c>
       <c r="AN19" s="4" t="n">
-        <v>21.76</v>
+        <v>3.56</v>
       </c>
       <c r="AO19" s="4" t="inlineStr">
         <is>
-          <t>T+1：冲到21.76先减仓，跌破19.75止损；若高开低走不恋战</t>
+          <t>T+1：冲到3.56先减仓，跌破3.23止损；若高开低走不恋战</t>
         </is>
       </c>
       <c r="AP19" s="4" t="n">
-        <v>19.04</v>
+        <v>3.12</v>
       </c>
       <c r="AQ19" s="4" t="n">
-        <v>22.19</v>
+        <v>3.63</v>
       </c>
       <c r="AR19" s="4" t="inlineStr">
         <is>
-          <t>T+2：未突破22.19且量能转弱则减仓，跌破19.04退出</t>
+          <t>T+2：未突破3.63且量能转弱则减仓，跌破3.12退出</t>
         </is>
       </c>
       <c r="AS19" s="4" t="n">
-        <v>19.14</v>
+        <v>3.12</v>
       </c>
       <c r="AT19" s="4" t="n">
-        <v>22.76</v>
+        <v>3.73</v>
       </c>
       <c r="AU19" s="4" t="inlineStr">
         <is>
-          <t>T+3：到22.76分批止盈，跌破19.14或MA5失守退出</t>
+          <t>T+3：到3.73分批止盈，跌破3.12或MA5失守退出</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4324,7 @@
         <v>3.91</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>85.58</v>
+        <v>83.78</v>
       </c>
       <c r="H20" s="4" t="n">
         <v>12.22</v>
@@ -4360,16 +4360,16 @@
         <v>5.62</v>
       </c>
       <c r="S20" s="4" t="n">
-        <v>0</v>
+        <v>-1.8</v>
       </c>
       <c r="T20" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>近期公告中性</t>
         </is>
       </c>
       <c r="U20" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额下降-1.0%</t>
         </is>
       </c>
       <c r="V20" s="4" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="W20" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>近期公告中性；融资余额下降-1.0%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X20" s="4" t="n">
@@ -4487,7 +4487,7 @@
         <v>8</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>82.56999999999999</v>
+        <v>83.37</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>5.4</v>
@@ -4523,16 +4523,16 @@
         <v>8.5</v>
       </c>
       <c r="S21" s="4" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="T21" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告</t>
+          <t>公告偏风险(1个负面关键词, 0个异动/风险词)</t>
         </is>
       </c>
       <c r="U21" s="4" t="inlineStr">
         <is>
-          <t>无两融数据</t>
+          <t>融资余额上升13.1%</t>
         </is>
       </c>
       <c r="V21" s="4" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="W21" s="4" t="inlineStr">
         <is>
-          <t>近期无重大公告；无两融数据；近期未上龙虎榜</t>
+          <t>公告偏风险(1个负面关键词, 0个异动/风险词)；融资余额上升13.1%；近期未上龙虎榜</t>
         </is>
       </c>
       <c r="X21" s="4" t="n">

</xml_diff>